<commit_message>
feat: 新增图鉴系统（DictionaryManager + DictionariesUI）
- 新增 DictionaryManager 管理物品/敌人解锁记录
- 新增 DictionariesUI 界面及 DictionaryItem/DictionarySlot 子项
- PlayerSaveData 新增 DiscoveredItemIds/DiscoveredEnemyIds 字段
- PlayerAccountDataManager 创建/加载存档时初始化图鉴
- EnemyEntityTable 新增 IconId 字段
- UIViews/UITable/ResourceConfigTable 注册图鉴相关资源
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/Core/UITable.xlsx
+++ b/AAAGameData/DataTables/Core/UITable.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="76">
   <si>
     <t>#</t>
   </si>
@@ -270,6 +270,12 @@
   </si>
   <si>
     <t>WarehouseUI</t>
+  </si>
+  <si>
+    <t>图鉴界面</t>
+  </si>
+  <si>
+    <t>DictionariesUI</t>
   </si>
 </sst>
 </file>
@@ -1234,7 +1240,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="13.1333333333333" customWidth="1"/>
@@ -1968,6 +1974,29 @@
         <v>1</v>
       </c>
       <c r="H34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="2:8">
+      <c r="B35">
+        <v>30</v>
+      </c>
+      <c r="C35" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35">
+        <v>2</v>
+      </c>
+      <c r="E35" t="s">
+        <v>75</v>
+      </c>
+      <c r="F35" t="b">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: BattlePresetUI Prefab 搭建 + UITable 注册
- BattlePresetUI Prefab 重新搭建，Variables 更新
- UIViews/UITable 注册出战预设UI
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/Core/UITable.xlsx
+++ b/AAAGameData/DataTables/Core/UITable.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="78">
   <si>
     <t>#</t>
   </si>
@@ -276,6 +276,12 @@
   </si>
   <si>
     <t>DictionariesUI</t>
+  </si>
+  <si>
+    <t>出战预设界面</t>
+  </si>
+  <si>
+    <t>BattlePresetUI</t>
   </si>
 </sst>
 </file>
@@ -1240,7 +1246,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="13.1333333333333" customWidth="1"/>
@@ -1997,6 +2003,29 @@
         <v>1</v>
       </c>
       <c r="H35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="2:8">
+      <c r="B36">
+        <v>31</v>
+      </c>
+      <c r="C36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36">
+        <v>2</v>
+      </c>
+      <c r="E36" t="s">
+        <v>77</v>
+      </c>
+      <c r="F36" t="b">
+        <v>0</v>
+      </c>
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 2: 配置表与数据管理器更新 (UITable, ResourceConfigTable, 数据管理器)
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/Core/UITable.xlsx
+++ b/AAAGameData/DataTables/Core/UITable.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11925"/>
+    <workbookView windowWidth="27948" windowHeight="11855"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="64">
   <si>
     <t>#</t>
   </si>
@@ -110,24 +110,6 @@
     <t>StartMenuUI</t>
   </si>
   <si>
-    <t>游戏界面</t>
-  </si>
-  <si>
-    <t>GameUIForm</t>
-  </si>
-  <si>
-    <t>游戏结算</t>
-  </si>
-  <si>
-    <t>GameOverUIForm</t>
-  </si>
-  <si>
-    <t>顶部资源栏</t>
-  </si>
-  <si>
-    <t>Topbar</t>
-  </si>
-  <si>
     <t>对话框(中层)</t>
   </si>
   <si>
@@ -135,30 +117,6 @@
   </si>
   <si>
     <t>SettingDialog</t>
-  </si>
-  <si>
-    <t>评分</t>
-  </si>
-  <si>
-    <t>RatingDialog</t>
-  </si>
-  <si>
-    <t>服务条款</t>
-  </si>
-  <si>
-    <t>TermsOfServiceDialog</t>
-  </si>
-  <si>
-    <t>通用提示对话框</t>
-  </si>
-  <si>
-    <t>CommonDialog</t>
-  </si>
-  <si>
-    <t>语言设置</t>
-  </si>
-  <si>
-    <t>LanguagesDialog</t>
   </si>
   <si>
     <t>提示(顶层)</t>
@@ -1246,12 +1204,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H36"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
+  <dimension ref="A1:H29"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="13.1333333333333" customWidth="1"/>
-    <col min="3" max="3" width="25.4416666666667" customWidth="1"/>
-    <col min="4" max="4" width="40.1333333333333" customWidth="1"/>
+    <col min="2" max="2" width="13.1296296296296" customWidth="1"/>
+    <col min="3" max="3" width="25.4444444444444" customWidth="1"/>
+    <col min="4" max="4" width="40.1296296296296" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="25.5" customWidth="1"/>
     <col min="7" max="7" width="10.5" customWidth="1"/>
@@ -1367,99 +1325,85 @@
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="A7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-      <c r="F7" t="b">
-        <v>1</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7" t="b">
-        <v>0</v>
-      </c>
+      <c r="C7" s="1"/>
+      <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:8">
       <c r="B8">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" t="b">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="1"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="B10">
+        <v>10</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10">
         <v>3</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8" t="s">
-        <v>23</v>
-      </c>
-      <c r="F8" t="b">
-        <v>1</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-      <c r="H8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="B9">
-        <v>4</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-      <c r="H9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:8">
       <c r="B11">
-        <v>5</v>
-      </c>
-      <c r="C11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11" t="s">
         <v>27</v>
       </c>
-      <c r="D11">
-        <v>1</v>
-      </c>
-      <c r="E11" t="s">
-        <v>28</v>
-      </c>
       <c r="F11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11">
         <v>2</v>
@@ -1470,22 +1414,22 @@
     </row>
     <row r="12" spans="1:8">
       <c r="B12">
-        <v>6</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>28</v>
       </c>
       <c r="D12">
         <v>2</v>
       </c>
-      <c r="E12" s="1" t="s">
-        <v>30</v>
+      <c r="E12" t="s">
+        <v>29</v>
       </c>
       <c r="F12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H12" t="b">
         <v>1</v>
@@ -1493,19 +1437,19 @@
     </row>
     <row r="13" spans="1:8">
       <c r="B13">
-        <v>7</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>31</v>
+        <v>13</v>
+      </c>
+      <c r="C13" t="s">
+        <v>30</v>
       </c>
       <c r="D13">
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G13">
         <v>2</v>
@@ -1516,22 +1460,22 @@
     </row>
     <row r="14" spans="1:8">
       <c r="B14">
-        <v>8</v>
-      </c>
-      <c r="C14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14" t="s">
         <v>33</v>
       </c>
-      <c r="D14">
+      <c r="F14" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14">
         <v>3</v>
-      </c>
-      <c r="E14" t="s">
-        <v>34</v>
-      </c>
-      <c r="F14" t="b">
-        <v>1</v>
-      </c>
-      <c r="G14">
-        <v>2</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
@@ -1539,41 +1483,55 @@
     </row>
     <row r="15" spans="1:8">
       <c r="B15">
-        <v>9</v>
-      </c>
-      <c r="C15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15" t="s">
         <v>35</v>
       </c>
-      <c r="D15">
-        <v>2</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="F15" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="B16">
+        <v>16</v>
+      </c>
+      <c r="C16" t="s">
         <v>36</v>
       </c>
-      <c r="F15" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15">
-        <v>2</v>
-      </c>
-      <c r="H15" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="1" t="s">
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="1"/>
-    </row>
-    <row r="17" spans="2:8">
+      <c r="F16" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="1" spans="2:8">
       <c r="B17">
-        <v>10</v>
-      </c>
-      <c r="C17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" t="s">
         <v>38</v>
       </c>
       <c r="D17">
@@ -1586,15 +1544,15 @@
         <v>0</v>
       </c>
       <c r="G17">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H17" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="2:8">
+    <row r="18" customFormat="1" spans="2:8">
       <c r="B18">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C18" t="s">
         <v>40</v>
@@ -1609,21 +1567,21 @@
         <v>0</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H18" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" customFormat="1" spans="2:8">
       <c r="B19">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s">
         <v>42</v>
       </c>
       <c r="D19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" t="s">
         <v>43</v>
@@ -1635,12 +1593,12 @@
         <v>1</v>
       </c>
       <c r="H19" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" customFormat="1" spans="2:8">
       <c r="B20">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="C20" t="s">
         <v>44</v>
@@ -1655,21 +1613,21 @@
         <v>0</v>
       </c>
       <c r="G20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:8">
       <c r="B21">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s">
         <v>46</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
         <v>47</v>
@@ -1678,7 +1636,7 @@
         <v>0</v>
       </c>
       <c r="G21">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H21" t="b">
         <v>0</v>
@@ -1686,7 +1644,7 @@
     </row>
     <row r="22" spans="2:8">
       <c r="B22">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="C22" t="s">
         <v>48</v>
@@ -1709,13 +1667,13 @@
     </row>
     <row r="23" spans="2:8">
       <c r="B23">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
         <v>50</v>
       </c>
       <c r="D23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E23" t="s">
         <v>51</v>
@@ -1727,24 +1685,24 @@
         <v>1</v>
       </c>
       <c r="H23" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="1" spans="2:8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8">
       <c r="B24">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
         <v>52</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E24" t="s">
         <v>53</v>
       </c>
       <c r="F24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1753,21 +1711,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" customFormat="1" spans="2:8">
+    <row r="25" spans="2:8">
       <c r="B25">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="C25" t="s">
         <v>54</v>
       </c>
       <c r="D25">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E25" t="s">
         <v>55</v>
       </c>
       <c r="F25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G25">
         <v>1</v>
@@ -1778,30 +1736,30 @@
     </row>
     <row r="26" customFormat="1" spans="2:8">
       <c r="B26">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="C26" t="s">
         <v>56</v>
       </c>
       <c r="D26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" t="s">
         <v>57</v>
       </c>
       <c r="F26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H26" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" customFormat="1" spans="2:8">
+    <row r="27" spans="2:8">
       <c r="B27">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C27" t="s">
         <v>58</v>
@@ -1819,12 +1777,12 @@
         <v>1</v>
       </c>
       <c r="H27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="2:8">
       <c r="B28">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="C28" t="s">
         <v>60</v>
@@ -1839,21 +1797,21 @@
         <v>0</v>
       </c>
       <c r="G28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="2:8">
       <c r="B29">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="C29" t="s">
         <v>62</v>
       </c>
       <c r="D29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E29" t="s">
         <v>63</v>
@@ -1865,167 +1823,6 @@
         <v>1</v>
       </c>
       <c r="H29" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="2:8">
-      <c r="B30">
-        <v>23</v>
-      </c>
-      <c r="C30" t="s">
-        <v>64</v>
-      </c>
-      <c r="D30">
-        <v>2</v>
-      </c>
-      <c r="E30" t="s">
-        <v>65</v>
-      </c>
-      <c r="F30" t="b">
-        <v>0</v>
-      </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-      <c r="H30" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="2:8">
-      <c r="B31">
-        <v>24</v>
-      </c>
-      <c r="C31" t="s">
-        <v>66</v>
-      </c>
-      <c r="D31">
-        <v>3</v>
-      </c>
-      <c r="E31" t="s">
-        <v>67</v>
-      </c>
-      <c r="F31" t="b">
-        <v>1</v>
-      </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-      <c r="H31" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="2:8">
-      <c r="B32">
-        <v>25</v>
-      </c>
-      <c r="C32" t="s">
-        <v>68</v>
-      </c>
-      <c r="D32">
-        <v>3</v>
-      </c>
-      <c r="E32" t="s">
-        <v>69</v>
-      </c>
-      <c r="F32" t="b">
-        <v>1</v>
-      </c>
-      <c r="G32">
-        <v>1</v>
-      </c>
-      <c r="H32" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="1" spans="2:8">
-      <c r="B33">
-        <v>28</v>
-      </c>
-      <c r="C33" t="s">
-        <v>70</v>
-      </c>
-      <c r="D33">
-        <v>2</v>
-      </c>
-      <c r="E33" t="s">
-        <v>71</v>
-      </c>
-      <c r="F33" t="b">
-        <v>1</v>
-      </c>
-      <c r="G33">
-        <v>2</v>
-      </c>
-      <c r="H33" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="2:8">
-      <c r="B34">
-        <v>29</v>
-      </c>
-      <c r="C34" t="s">
-        <v>72</v>
-      </c>
-      <c r="D34">
-        <v>2</v>
-      </c>
-      <c r="E34" t="s">
-        <v>73</v>
-      </c>
-      <c r="F34" t="b">
-        <v>0</v>
-      </c>
-      <c r="G34">
-        <v>1</v>
-      </c>
-      <c r="H34" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="2:8">
-      <c r="B35">
-        <v>30</v>
-      </c>
-      <c r="C35" t="s">
-        <v>74</v>
-      </c>
-      <c r="D35">
-        <v>2</v>
-      </c>
-      <c r="E35" t="s">
-        <v>75</v>
-      </c>
-      <c r="F35" t="b">
-        <v>0</v>
-      </c>
-      <c r="G35">
-        <v>1</v>
-      </c>
-      <c r="H35" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="2:8">
-      <c r="B36">
-        <v>31</v>
-      </c>
-      <c r="C36" t="s">
-        <v>76</v>
-      </c>
-      <c r="D36">
-        <v>2</v>
-      </c>
-      <c r="E36" t="s">
-        <v>77</v>
-      </c>
-      <c r="F36" t="b">
-        <v>0</v>
-      </c>
-      <c r="G36">
-        <v>1</v>
-      </c>
-      <c r="H36" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2040,7 +1837,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -2051,7 +1848,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>

<commit_message>
feat: 宝箱UI系统 — TreasureBoxUI 完整实现
新增宝箱界面（TreasureBoxUI）及其数据载体、容器实现，
TreasureChestInteractable 对接打开宝箱UI逻辑，
InventorySlotUI 支持宝箱容器上下文菜单
</commit_message>
<xml_diff>
--- a/AAAGameData/DataTables/Core/UITable.xlsx
+++ b/AAAGameData/DataTables/Core/UITable.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27948" windowHeight="11855"/>
+    <workbookView windowWidth="28800" windowHeight="11925"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="66">
   <si>
     <t>#</t>
   </si>
@@ -240,6 +240,12 @@
   </si>
   <si>
     <t>BattlePresetUI</t>
+  </si>
+  <si>
+    <t>宝箱界面</t>
+  </si>
+  <si>
+    <t>TreasureBoxUI</t>
   </si>
 </sst>
 </file>
@@ -1204,12 +1210,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <dimension ref="A1:H30"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="13.1296296296296" customWidth="1"/>
-    <col min="3" max="3" width="25.4444444444444" customWidth="1"/>
-    <col min="4" max="4" width="40.1296296296296" customWidth="1"/>
+    <col min="2" max="2" width="13.1333333333333" customWidth="1"/>
+    <col min="3" max="3" width="25.4416666666667" customWidth="1"/>
+    <col min="4" max="4" width="40.1333333333333" customWidth="1"/>
     <col min="5" max="5" width="23" customWidth="1"/>
     <col min="6" max="6" width="25.5" customWidth="1"/>
     <col min="7" max="7" width="10.5" customWidth="1"/>
@@ -1823,6 +1829,29 @@
         <v>1</v>
       </c>
       <c r="H29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="2:8">
+      <c r="B30">
+        <v>32</v>
+      </c>
+      <c r="C30" t="s">
+        <v>64</v>
+      </c>
+      <c r="D30">
+        <v>2</v>
+      </c>
+      <c r="E30" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" t="b">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1837,7 +1866,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>
@@ -1848,7 +1877,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>